<commit_message>
Updated allrue Report changes and Jenkins file changes
</commit_message>
<xml_diff>
--- a/Data Files/Create New User2.xlsx
+++ b/Data Files/Create New User2.xlsx
@@ -544,7 +544,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:T4"/>
+  <dimension ref="A1:S4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" bestFit="true" customWidth="true" width="11.7109375" collapsed="true"/>
@@ -557,221 +557,221 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19">
-      <c r="A1" t="s">
+      <c r="A1" t="s" s="0">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" t="s" s="0">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" t="s" s="0">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" t="s" s="0">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" t="s" s="0">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" t="s" s="0">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" t="s" s="0">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" t="s" s="0">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" t="s" s="0">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" t="s" s="0">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" t="s" s="0">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" t="s" s="0">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" t="s" s="0">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" t="s" s="0">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" t="s" s="0">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" t="s" s="0">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" t="s" s="0">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" t="s" s="0">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" t="s" s="0">
         <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:19">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>19</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>20</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" t="s" s="0">
         <v>22</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" t="s" s="0">
         <v>23</v>
       </c>
-      <c r="F2">
+      <c r="F2" s="0">
         <v>14</v>
       </c>
-      <c r="G2">
+      <c r="G2" s="0">
         <v>8</v>
       </c>
-      <c r="H2">
+      <c r="H2" s="0">
         <v>1992</v>
       </c>
-      <c r="I2" t="s">
+      <c r="I2" t="s" s="0">
         <v>24</v>
       </c>
-      <c r="J2" t="s">
+      <c r="J2" t="s" s="0">
         <v>25</v>
       </c>
-      <c r="K2" t="s">
+      <c r="K2" t="s" s="0">
         <v>26</v>
       </c>
-      <c r="L2" t="s">
+      <c r="L2" t="s" s="0">
         <v>27</v>
       </c>
-      <c r="N2" t="s">
+      <c r="N2" t="s" s="0">
         <v>28</v>
       </c>
-      <c r="O2">
+      <c r="O2" s="0">
         <v>421503</v>
       </c>
-      <c r="P2" t="s">
+      <c r="P2" t="s" s="0">
         <v>29</v>
       </c>
-      <c r="Q2" t="s">
+      <c r="Q2" t="s" s="0">
         <v>30</v>
       </c>
-      <c r="R2">
+      <c r="R2" s="0">
         <v>9999999999</v>
       </c>
-      <c r="S2" t="s">
+      <c r="S2" t="s" s="0">
         <v>47</v>
       </c>
     </row>
     <row r="3" spans="1:19">
-      <c r="A3" t="s">
+      <c r="A3" t="s" s="0">
         <v>31</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" t="s" s="0">
         <v>32</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" t="s" s="0">
         <v>34</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" t="s" s="0">
         <v>23</v>
       </c>
-      <c r="F3">
+      <c r="F3" s="0">
         <v>23</v>
       </c>
-      <c r="G3">
+      <c r="G3" s="0">
         <v>7</v>
       </c>
-      <c r="H3">
+      <c r="H3" s="0">
         <v>1995</v>
       </c>
-      <c r="I3" t="s">
+      <c r="I3" t="s" s="0">
         <v>35</v>
       </c>
-      <c r="J3" t="s">
+      <c r="J3" t="s" s="0">
         <v>36</v>
       </c>
-      <c r="K3" t="s">
+      <c r="K3" t="s" s="0">
         <v>37</v>
       </c>
-      <c r="L3" t="s">
+      <c r="L3" t="s" s="0">
         <v>38</v>
       </c>
-      <c r="N3" t="s">
+      <c r="N3" t="s" s="0">
         <v>28</v>
       </c>
-      <c r="O3">
+      <c r="O3" s="0">
         <v>420086</v>
       </c>
-      <c r="P3" t="s">
+      <c r="P3" t="s" s="0">
         <v>39</v>
       </c>
-      <c r="Q3" t="s">
+      <c r="Q3" t="s" s="0">
         <v>40</v>
       </c>
-      <c r="R3">
+      <c r="R3" s="0">
         <v>8888888888</v>
       </c>
-      <c r="S3" t="s">
+      <c r="S3" t="s" s="0">
         <v>47</v>
       </c>
     </row>
     <row r="4" spans="1:19">
-      <c r="A4" t="s">
+      <c r="A4" t="s" s="0">
         <v>41</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" t="s" s="0">
         <v>42</v>
       </c>
       <c r="C4" s="1"/>
-      <c r="E4" t="s">
+      <c r="E4" t="s" s="0">
         <v>23</v>
       </c>
-      <c r="F4">
+      <c r="F4" s="0">
         <v>11</v>
       </c>
-      <c r="G4">
+      <c r="G4" s="0">
         <v>11</v>
       </c>
-      <c r="H4">
+      <c r="H4" s="0">
         <v>2011</v>
       </c>
-      <c r="I4" t="s">
+      <c r="I4" t="s" s="0">
         <v>43</v>
       </c>
-      <c r="J4" t="s">
+      <c r="J4" t="s" s="0">
         <v>44</v>
       </c>
-      <c r="K4" t="s">
+      <c r="K4" t="s" s="0">
         <v>45</v>
       </c>
-      <c r="N4" t="s">
+      <c r="N4" t="s" s="0">
         <v>28</v>
       </c>
-      <c r="O4">
+      <c r="O4" s="0">
         <v>4200078</v>
       </c>
-      <c r="P4" t="s">
+      <c r="P4" t="s" s="0">
         <v>29</v>
       </c>
-      <c r="Q4" t="s">
+      <c r="Q4" t="s" s="0">
         <v>46</v>
       </c>
-      <c r="R4">
+      <c r="R4" s="0">
         <v>7070707070</v>
       </c>
-      <c r="S4" t="s">
+      <c r="S4" t="s" s="0">
         <v>47</v>
       </c>
     </row>

</xml_diff>